<commit_message>
Auto update: 2026-02-24 22:00:35
</commit_message>
<xml_diff>
--- a/股价记录.xlsx
+++ b/股价记录.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1412,6 +1412,513 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:51:20</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E25" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F25" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G25" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H25" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I25" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:01:24</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E26" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F26" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G26" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H26" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I26" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:11:29</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D27" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E27" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F27" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G27" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H27" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I27" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:21:41</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E28" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F28" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G28" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H28" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I28" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:31:47</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E29" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F29" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G29" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H29" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I29" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:41:52</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D30" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E30" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F30" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G30" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H30" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I30" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:52:00</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D31" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E31" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F31" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G31" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H31" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I31" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:02:11</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D32" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E32" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F32" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G32" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H32" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I32" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:12:18</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E33" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F33" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G33" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H33" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I33" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:22:24</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D34" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E34" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F34" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G34" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H34" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I34" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:32:29</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D35" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E35" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F35" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G35" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H35" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I35" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:42:34</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D36" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E36" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F36" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G36" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H36" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I36" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:52:38</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>17.72</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="E37" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="F37" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="G37" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="H37" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I37" t="n">
+        <v>57298600</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1014180787</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1423,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2290,6 +2797,513 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:51:20</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C24" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E24" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F24" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G24" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H24" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I24" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:01:24</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C25" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E25" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F25" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G25" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H25" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I25" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:11:29</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C26" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E26" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F26" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G26" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H26" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I26" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:21:41</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C27" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E27" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F27" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G27" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H27" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I27" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:31:47</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C28" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E28" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F28" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G28" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H28" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I28" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:41:52</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C29" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E29" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F29" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G29" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H29" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I29" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:52:00</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C30" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E30" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F30" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G30" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H30" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I30" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:02:11</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C31" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E31" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F31" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G31" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H31" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I31" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:12:19</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C32" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E32" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F32" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G32" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H32" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I32" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:22:24</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C33" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E33" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F33" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G33" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H33" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I33" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:32:29</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C34" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E34" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F34" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G34" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H34" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I34" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:42:34</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C35" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E35" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F35" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G35" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H35" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I35" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:52:38</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="C36" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="E36" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="F36" t="n">
+        <v>18.59</v>
+      </c>
+      <c r="G36" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="H36" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="I36" t="n">
+        <v>81562500</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1503552137</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2301,7 +3315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3163,6 +4177,513 @@
         <v>636759332</v>
       </c>
       <c r="K23" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:51:20</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E24" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G24" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H24" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I24" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J24" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:01:24</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E25" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G25" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H25" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I25" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J25" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:11:29</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E26" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G26" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H26" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I26" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J26" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:21:41</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E27" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G27" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H27" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I27" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J27" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:31:47</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E28" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G28" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H28" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I28" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J28" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:41:53</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E29" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G29" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H29" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I29" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J29" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:52:00</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E30" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G30" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H30" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I30" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J30" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:02:12</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E31" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G31" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H31" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I31" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J31" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:12:19</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E32" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G32" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H32" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I32" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J32" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:22:24</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E33" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G33" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H33" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I33" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J33" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:32:30</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E34" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G34" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H34" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I34" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J34" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:42:35</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E35" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G35" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H35" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I35" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J35" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:52:39</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E36" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="G36" t="n">
+        <v>18.98</v>
+      </c>
+      <c r="H36" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I36" t="n">
+        <v>33379900</v>
+      </c>
+      <c r="J36" t="n">
+        <v>636759332</v>
+      </c>
+      <c r="K36" t="inlineStr">
         <is>
           <t>实时查询</t>
         </is>
@@ -10712,7 +12233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11579,6 +13100,513 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:51:20</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E24" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F24" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G24" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H24" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I24" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J24" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:01:23</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E25" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F25" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G25" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H25" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I25" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J25" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:11:29</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E26" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F26" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G26" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H26" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I26" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J26" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:21:40</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D27" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E27" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F27" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G27" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H27" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I27" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J27" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:31:46</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E28" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F28" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G28" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H28" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I28" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J28" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:41:52</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E29" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F29" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G29" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H29" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I29" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J29" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-24 20:52:00</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D30" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E30" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F30" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G30" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H30" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I30" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J30" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:02:11</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D31" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E31" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F31" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G31" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H31" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I31" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J31" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:12:18</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D32" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E32" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F32" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G32" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H32" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I32" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J32" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:22:23</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E33" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F33" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G33" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H33" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I33" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J33" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:32:29</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D34" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E34" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F34" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G34" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H34" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I34" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J34" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:42:34</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D35" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E35" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F35" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G35" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H35" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I35" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J35" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-02-24 21:52:38</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D36" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="E36" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F36" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="G36" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H36" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="I36" t="n">
+        <v>52349100</v>
+      </c>
+      <c r="J36" t="n">
+        <v>642162306</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>实时查询</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>